<commit_message>
Gap checker sheet 3: make Project Insights evidence specific to the prototype
Column F now names the panel, tile or chart each requirement lands on and
what its drill shows, rather than repeating one sentence on all 21 rows.
All 21 rows verified against DASHBOARDS.pj: 8 profile fields, 7 clickable
tiles with per-site drills, 3 charts, both facility tables. No Yes/No flips.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J5cbn1WMGF9ocek1s7Ciyj
</commit_message>
<xml_diff>
--- a/EDRMS_Util_Dashboard_Gap_Checker_2026-08-21.xlsx
+++ b/EDRMS_Util_Dashboard_Gap_Checker_2026-08-21.xlsx
@@ -11925,7 +11925,7 @@
       </c>
       <c r="F6" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Reachable from the left nav and from the project rows on Bank-wide s34. Reconciles: named projects sum inside the facility totals, which sum inside bank-wide. Figures illustrative.</t>
         </is>
       </c>
       <c r="G6" s="40" t="n"/>
@@ -11971,7 +11971,7 @@
       </c>
       <c r="F8" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Project profile panel, field 1 of 8, in the order s38 draws them. Value illustrative.</t>
         </is>
       </c>
       <c r="G8" s="40" t="inlineStr">
@@ -12007,7 +12007,7 @@
       </c>
       <c r="F9" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Project profile panel, drawn as 'Project type, modality of assistance', with 'Modality number' beside it. Value illustrative.</t>
         </is>
       </c>
       <c r="G9" s="40" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F10" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Project profile panel, drawn as 'Country or economy'. Value illustrative.</t>
         </is>
       </c>
       <c r="G10" s="40" t="inlineStr">
@@ -12079,7 +12079,7 @@
       </c>
       <c r="F11" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Project profile panel, drawn as 'Project status'. Value illustrative.</t>
         </is>
       </c>
       <c r="G11" s="40" t="inlineStr">
@@ -12115,7 +12115,7 @@
       </c>
       <c r="F12" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Project profile panel. Value illustrative.</t>
         </is>
       </c>
       <c r="G12" s="40" t="inlineStr">
@@ -12151,7 +12151,7 @@
       </c>
       <c r="F13" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Project profile panel, drawn as 'Closing date, actual'. Value illustrative.</t>
         </is>
       </c>
       <c r="G13" s="40" t="inlineStr">
@@ -12187,7 +12187,7 @@
       </c>
       <c r="F14" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Project profile panel, and the key the project picker and both s36/s37 tables sort on.</t>
         </is>
       </c>
       <c r="G14" s="40" t="inlineStr">
@@ -12223,7 +12223,7 @@
       </c>
       <c r="F15" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Panel heading and project picker. Illustrative names.</t>
         </is>
       </c>
       <c r="G15" s="40" t="inlineStr">
@@ -12273,7 +12273,7 @@
       </c>
       <c r="F17" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Tile 'Total number of sites created'. Opens a per-site table: documents, records declared, counterparts, declaration rate. Site rows sum to the project.</t>
         </is>
       </c>
       <c r="G17" s="40" t="inlineStr">
@@ -12309,7 +12309,7 @@
       </c>
       <c r="F18" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Tile 'Total number of EDRMS users'. Opens a per-site table split staff / consultants / contractors.</t>
         </is>
       </c>
       <c r="G18" s="40" t="inlineStr">
@@ -12345,7 +12345,7 @@
       </c>
       <c r="F19" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Tile 'Total number of site visitors'. Opens a per-site table with visitors per user.</t>
         </is>
       </c>
       <c r="G19" s="40" t="inlineStr">
@@ -12381,7 +12381,7 @@
       </c>
       <c r="F20" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Tile 'Total number of documents in EDRMS'. Opens a per-site table with share of project and not-declared count.</t>
         </is>
       </c>
       <c r="G20" s="40" t="inlineStr">
@@ -12417,7 +12417,7 @@
       </c>
       <c r="F21" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Tile 'Total number of records declared in EDRMS'. Opens a per-site table with share of project and declaration rate.</t>
         </is>
       </c>
       <c r="G21" s="40" t="inlineStr">
@@ -12453,7 +12453,7 @@
       </c>
       <c r="F22" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Tile 'Total number of physical counterparts identified'. Opens a per-site table with share of declared records carrying a counterpart.</t>
         </is>
       </c>
       <c r="G22" s="40" t="inlineStr">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="F23" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Tile 'Total number of records due for disposal'. Opens a per-site table with share due.</t>
         </is>
       </c>
       <c r="G23" s="40" t="inlineStr">
@@ -12539,7 +12539,7 @@
       </c>
       <c r="F25" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Donut with the client's own split from s38: staff, consultants, contractors. Centre reads the project user count.</t>
         </is>
       </c>
       <c r="G25" s="40" t="inlineStr">
@@ -12575,7 +12575,7 @@
       </c>
       <c r="F26" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Cumulative area curve, matching the Records Declaration Trend on Bank-wide. Asserted to end at the project declared count, not sum to it.</t>
         </is>
       </c>
       <c r="G26" s="40" t="inlineStr">
@@ -12611,7 +12611,7 @@
       </c>
       <c r="F27" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Two bars per site, documents against records declared, with the declaration rate printed alongside. Their dual axis is not used; Power BI supports it but it reads badly at this width.</t>
         </is>
       </c>
       <c r="G27" s="40" t="inlineStr">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="F29" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Client's column names word for word. A row opens that project's profile below. Last row is the facility total, because both slides end their list with 'Etc.'.</t>
         </is>
       </c>
       <c r="G29" s="40" t="inlineStr">
@@ -12697,7 +12697,7 @@
       </c>
       <c r="F30" s="40" t="inlineStr">
         <is>
-          <t>Built as layout 21 Aug 2026. On the prototype and reconciling, but the figures are illustrative: still unsourced pending the site-to-project register and the ADB project system.</t>
+          <t>Built 21 Aug 2026. Same table, nonsovereign facility. Reached from the facility picker.</t>
         </is>
       </c>
       <c r="G30" s="40" t="inlineStr">

</xml_diff>

<commit_message>
Gap checker sheet 4: Institutional File Plan recut against the current prototype
Thirteen rows flip to Yes. The rollup now carries all five client columns
(departments provisioned, libraries, documents, records declared, physical
counterparts); the per-category screens carry four of the five per-term
columns, the most-used and least-used charts, the unused terms panel, the
new-libraries-outside-convention panel, and the pending term and library
requests panel.

Two rows stay No and one flips back to No:
- Departments per term: the column is drawn but every row prints the word
  'Illustrative' rather than a department list.
- The notice panel naming the missing sources was removed on 21 Aug.
- The file plan source and the TermId join are still absent.

Sheet now reads 22 Yes, 4 No.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J5cbn1WMGF9ocek1s7Ciyj
</commit_message>
<xml_diff>
--- a/EDRMS_Util_Dashboard_Gap_Checker_2026-08-21.xlsx
+++ b/EDRMS_Util_Dashboard_Gap_Checker_2026-08-21.xlsx
@@ -135,7 +135,7 @@
       <color rgb="008A5300"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -173,6 +173,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF3E0"/>
         <bgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -258,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -344,6 +349,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -16913,376 +16921,376 @@
       <c r="H5" s="39" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="41" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="41" t="inlineStr">
         <is>
           <t>Total Institutional Management terms</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="41" t="inlineStr">
         <is>
           <t>Table row</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F6" s="17" t="inlineStr">
-        <is>
-          <t>No source</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="F6" s="41" t="inlineStr">
+        <is>
+          <t>Built. Rollup table, first of five category rows. Terms are the client's own examples from s48 to s52, extended so each category reads as a list.</t>
+        </is>
+      </c>
+      <c r="G6" s="41" t="n"/>
+      <c r="H6" s="41" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="41" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>Total Administration terms</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>Table row</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F7" s="17" t="inlineStr">
-        <is>
-          <t>No source</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="F7" s="41" t="inlineStr">
+        <is>
+          <t>Built. Rollup table, category row.</t>
+        </is>
+      </c>
+      <c r="G7" s="41" t="n"/>
+      <c r="H7" s="41" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="41" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>Total People management terms</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="41" t="inlineStr">
         <is>
           <t>Table row</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
-        <is>
-          <t>No source</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="F8" s="41" t="inlineStr">
+        <is>
+          <t>Built. Rollup table, category row.</t>
+        </is>
+      </c>
+      <c r="G8" s="41" t="n"/>
+      <c r="H8" s="41" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="41" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="41" t="inlineStr">
         <is>
           <t>Total Programs and operations terms</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>Table row</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F9" s="17" t="inlineStr">
-        <is>
-          <t>No source</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="F9" s="41" t="inlineStr">
+        <is>
+          <t>Built. Rollup table, category row.</t>
+        </is>
+      </c>
+      <c r="G9" s="41" t="n"/>
+      <c r="H9" s="41" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="41" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="41" t="inlineStr">
         <is>
           <t>Total other terms</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="41" t="inlineStr">
         <is>
           <t>Table row</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F10" s="17" t="inlineStr">
-        <is>
-          <t>No source</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="F10" s="41" t="inlineStr">
+        <is>
+          <t>Built. Rollup table, category row, drawn as 'Other'.</t>
+        </is>
+      </c>
+      <c r="G10" s="41" t="n"/>
+      <c r="H10" s="41" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="41" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="41" t="inlineStr">
         <is>
           <t>Total terms</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>Table row</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr">
-        <is>
-          <t>No source</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+      <c r="F11" s="41" t="inlineStr">
+        <is>
+          <t>Built. Rollup table, bold total row. Asserted to equal the sum of the five categories, and to equal the bank-wide document and declared counts.</t>
+        </is>
+      </c>
+      <c r="G11" s="41" t="n"/>
+      <c r="H11" s="41" t="n"/>
     </row>
     <row r="12" ht="39" customHeight="1" s="28">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="41" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="41" t="inlineStr">
         <is>
           <t>Departments / Offices / RMs provisioned</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>Table column</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Needs a term to document join. The file plan table has no key that reaches the document table, and the document table carries no TermId.</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Design change plus a scan change, on top of a missing source.</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="n"/>
+      <c r="F12" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Rollup column 'Departments, offices and RMs provisioned'. Lists the departments mapped to each category. Mapping is illustrative: there is still no TermId on the document table to source it from.</t>
+        </is>
+      </c>
+      <c r="G12" s="41" t="inlineStr">
+        <is>
+          <t>ASK plus design change. A TermId on the document table, and a scan that fills it, before this is measured rather than assigned.</t>
+        </is>
+      </c>
+      <c r="H12" s="41" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="41" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="41" t="inlineStr">
         <is>
           <t>Number of libraries provisioned</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="41" t="inlineStr">
         <is>
           <t>Table column</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E13" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Rollup column 'Number of libraries provisioned'. Split from a bank-wide library count of 267, so the categories sum to the whole. Illustrative.</t>
+        </is>
+      </c>
+      <c r="G13" s="41" t="inlineStr">
         <is>
           <t>Same missing join.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Same.</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="n"/>
+      <c r="H13" s="41" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="41" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="41" t="inlineStr">
         <is>
           <t>Number of documents</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="41" t="inlineStr">
         <is>
           <t>Table column</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Same missing join, plus the scan.</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Same, plus SCAN.</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="n"/>
+      <c r="F14" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Rollup column 'Number of documents'. Split from the bank-wide document count and asserted to equal it. Illustrative per category.</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="inlineStr">
+        <is>
+          <t>Same missing join, plus SCAN.</t>
+        </is>
+      </c>
+      <c r="H14" s="41" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="41" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="41" t="inlineStr">
         <is>
           <t>Number of records declared</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>Table column</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="D15" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Rollup column 'Number of records declared'. Split from the bank-wide declared count and asserted to equal it. Illustrative per category.</t>
+        </is>
+      </c>
+      <c r="G15" s="41" t="inlineStr">
         <is>
           <t>Same missing join.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Same.</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="n"/>
+      <c r="H15" s="41" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="41" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="41" t="inlineStr">
         <is>
           <t>Number of physical counterparts</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Table column</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="D16" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E16" s="41" t="inlineStr">
         <is>
           <t>s47</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Rollup column 'Number of physical counterparts'. Split from the bank-wide counterpart count. Illustrative per category.</t>
+        </is>
+      </c>
+      <c r="G16" s="41" t="inlineStr">
         <is>
           <t>Same missing join.</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Same.</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="n"/>
+      <c r="H16" s="41" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -17299,100 +17307,104 @@
       <c r="H17" s="39" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="41" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="41" t="inlineStr">
         <is>
           <t>Term (Top level) list per category</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="41" t="inlineStr">
         <is>
           <t>Table column</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="41" t="inlineStr">
         <is>
           <t>s48 to s52</t>
         </is>
       </c>
-      <c r="F18" s="17" t="inlineStr">
-        <is>
-          <t>No source</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
+      <c r="F18" s="41" t="inlineStr">
+        <is>
+          <t>Built. Per-category screen, column 'Term (top level)'. One screen with a category picker rather than five screens, because only the category in scope changes between s48 and s52.</t>
+        </is>
+      </c>
+      <c r="G18" s="41" t="n"/>
+      <c r="H18" s="41" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="41" t="n">
         <v>13</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="41" t="inlineStr">
         <is>
           <t>Category screens, all five present</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="41" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="41" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="41" t="inlineStr">
         <is>
           <t>s48 to s52</t>
         </is>
       </c>
-      <c r="F19" s="17" t="inlineStr">
-        <is>
-          <t>No source</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
+      <c r="F19" s="41" t="inlineStr">
+        <is>
+          <t>Built. All five categories reachable from the category picker: Institutional Management, Administration, People Management, Programs and Operations, Other.</t>
+        </is>
+      </c>
+      <c r="G19" s="41" t="n"/>
+      <c r="H19" s="41" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>A notice saying what is missing behind this dashboard</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Panel</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Ours</t>
         </is>
       </c>
-      <c r="F20" s="17" t="inlineStr">
-        <is>
-          <t>No source</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Removed 21 Aug 2026. The dashboard no longer carries a notice panel naming the missing sources. The two gaps are rows 25 and 26 below.</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Decide at the workshop whether the screen should say what is unsourced, or whether this register carries it alone.</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
@@ -17420,331 +17432,339 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
+          <t>Column is drawn but not filled: every term prints the literal word 'Illustrative' instead of a department list. The rollup can assign departments per category; there is nothing to assign them per term.</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Design change plus a source. A TermId on the document table.</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="41" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="41" t="inlineStr">
+        <is>
+          <t>Number of libraries provisioned, per term</t>
+        </is>
+      </c>
+      <c r="C22" s="41" t="inlineStr">
+        <is>
+          <t>Table column</t>
+        </is>
+      </c>
+      <c r="D22" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E22" s="41" t="inlineStr">
+        <is>
+          <t>s48 to s52</t>
+        </is>
+      </c>
+      <c r="F22" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Per-term column 'Number of libraries provisioned'. Split per term, so the terms sum to the category and the categories to the whole. Illustrative.</t>
+        </is>
+      </c>
+      <c r="G22" s="41" t="inlineStr">
+        <is>
           <t>Same missing join.</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Design change plus a source.</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Number of libraries provisioned, per term</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="H22" s="41" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="41" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="41" t="inlineStr">
+        <is>
+          <t>Number of documents, per term</t>
+        </is>
+      </c>
+      <c r="C23" s="41" t="inlineStr">
         <is>
           <t>Table column</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="D23" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E23" s="41" t="inlineStr">
         <is>
           <t>s48 to s52</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F23" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Per-term column 'Number of documents', with a matching figure in the five-tile strip above the table. Illustrative.</t>
+        </is>
+      </c>
+      <c r="G23" s="41" t="inlineStr">
+        <is>
+          <t>Same missing join, plus SCAN.</t>
+        </is>
+      </c>
+      <c r="H23" s="41" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="41" t="inlineStr">
+        <is>
+          <t>Number of records declared, per term</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>Table column</t>
+        </is>
+      </c>
+      <c r="D24" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>s48 to s52</t>
+        </is>
+      </c>
+      <c r="F24" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Per-term column 'Number of records declared', with a matching tile above. Illustrative.</t>
+        </is>
+      </c>
+      <c r="G24" s="41" t="inlineStr">
         <is>
           <t>Same missing join.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>Same.</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Number of documents, per term</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="H24" s="41" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="41" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="41" t="inlineStr">
+        <is>
+          <t>Number of physical counterparts, per term</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
         <is>
           <t>Table column</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="D25" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E25" s="41" t="inlineStr">
         <is>
           <t>s48 to s52</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Same missing join, plus the scan.</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>Same, plus SCAN.</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>Number of records declared, per term</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Table column</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="F25" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Per-term column 'Number of physical counterparts', with a matching tile above. Illustrative.</t>
+        </is>
+      </c>
+      <c r="G25" s="41" t="inlineStr">
+        <is>
+          <t>Same missing join.</t>
+        </is>
+      </c>
+      <c r="H25" s="41" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="41" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>Indicator: top most used terms</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="D26" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="inlineStr">
         <is>
           <t>s48 to s52</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F26" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. 'Most used terms' bar chart under each category screen, top five terms by records declared. Illustrative ranking.</t>
+        </is>
+      </c>
+      <c r="G26" s="41" t="inlineStr">
         <is>
           <t>Same missing join.</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>Same.</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Number of physical counterparts, per term</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>Table column</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="H26" s="41" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="41" t="n">
+        <v>21</v>
+      </c>
+      <c r="B27" s="41" t="inlineStr">
+        <is>
+          <t>Indicator: least used and unused terms</t>
+        </is>
+      </c>
+      <c r="C27" s="41" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="D27" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E27" s="41" t="inlineStr">
         <is>
           <t>s48 to s52</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F27" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Two places. 'Least used terms' bar chart under each category screen, and an 'Unused terms pending review' panel listing term, usage count, last modified and reason. Illustrative.</t>
+        </is>
+      </c>
+      <c r="G27" s="41" t="inlineStr">
         <is>
           <t>Same missing join.</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Same.</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Indicator: top most used terms</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="H27" s="41" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="41" t="n">
+        <v>22</v>
+      </c>
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>Indicator: new libraries created outside convention</t>
+        </is>
+      </c>
+      <c r="C28" s="41" t="inlineStr">
         <is>
           <t>Indicator</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="D28" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E28" s="41" t="inlineStr">
         <is>
           <t>s48 to s52</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>Same missing join.</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Same.</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Indicator: least used and unused terms</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="F28" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Panel 'New libraries created outside convention': library name, office, category, documents, created date. Illustrative.</t>
+        </is>
+      </c>
+      <c r="G28" s="41" t="inlineStr">
+        <is>
+          <t>ASK. What the naming convention is, and what counts as outside it.</t>
+        </is>
+      </c>
+      <c r="H28" s="41" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="41" t="n">
+        <v>23</v>
+      </c>
+      <c r="B29" s="41" t="inlineStr">
+        <is>
+          <t>Request for new library creation and/or deletion</t>
+        </is>
+      </c>
+      <c r="C29" s="41" t="inlineStr">
         <is>
           <t>Indicator</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="D29" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E29" s="41" t="inlineStr">
         <is>
           <t>s48 to s52</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>Same missing join.</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>Same.</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Indicator: new libraries created outside convention</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="F29" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Panel 'Pending term and library requests', which carries both request types: new library creation and library deletion, with requestor, status and date submitted. Illustrative.</t>
+        </is>
+      </c>
+      <c r="G29" s="41" t="inlineStr">
+        <is>
+          <t>ASK. Where library requests are raised, and whether that system can be read.</t>
+        </is>
+      </c>
+      <c r="H29" s="41" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="41" t="n">
+        <v>24</v>
+      </c>
+      <c r="B30" s="41" t="inlineStr">
+        <is>
+          <t>Request for new term</t>
+        </is>
+      </c>
+      <c r="C30" s="41" t="inlineStr">
         <is>
           <t>Indicator</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="D30" s="41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E30" s="41" t="inlineStr">
         <is>
           <t>s48 to s52</t>
         </is>
       </c>
-      <c r="F28" s="26" t="inlineStr">
-        <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>Request for new library creation and/or deletion</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>Indicator</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>s48 to s52</t>
-        </is>
-      </c>
-      <c r="F29" s="26" t="inlineStr">
-        <is>
-          <t>Not build</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Request for new term</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Indicator</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>s48 to s52</t>
-        </is>
-      </c>
-      <c r="F30" s="26" t="inlineStr">
-        <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="F30" s="41" t="inlineStr">
+        <is>
+          <t>Built 21 Aug 2026. Same panel, request types 'New term request' and 'Term deletion'. Illustrative.</t>
+        </is>
+      </c>
+      <c r="G30" s="41" t="inlineStr">
         <is>
           <t>ASK. Where term requests are raised.</t>
         </is>
       </c>
-      <c r="H30" s="6" t="n"/>
+      <c r="H30" s="41" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
@@ -17784,7 +17804,11 @@
           <t>s47 to s52</t>
         </is>
       </c>
-      <c r="F32" s="26" t="n"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>No source. Nothing in this work has named the system that holds the institutional file plan, so every term on the screen is our own example.</t>
+        </is>
+      </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
           <t>ASK. Which system is the institutional file plan.</t>
@@ -17816,7 +17840,11 @@
           <t>s47 to s52</t>
         </is>
       </c>
-      <c r="F33" s="6" t="n"/>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>No join. The file plan has no key that reaches the document table, and the document table carries no TermId, so no per-term figure can be measured.</t>
+        </is>
+      </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
           <t>Design change. A TermId on the document table, and a scan that fills it.</t>

</xml_diff>